<commit_message>
create chart for data vizualization for ELNINO
</commit_message>
<xml_diff>
--- a/ELNINO DATA ANALYSIS IN KENYA.xlsx
+++ b/ELNINO DATA ANALYSIS IN KENYA.xlsx
@@ -8,20 +8,40 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Hi!\Documents\Dataanalytics\Projects\Excel\ELNINO-DATA-RESEARCH-AND-ANALYSIS-IN-KENYA\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5600233E-8B57-4A00-A814-3E4E89E794C3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B0722B21-74CA-430F-81B0-74D77BE53F20}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet2" sheetId="2" r:id="rId1"/>
     <sheet name="Sheet1" sheetId="1" r:id="rId2"/>
+    <sheet name="Sheet3" sheetId="3" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlcn.WorksheetConnection_Sheet1A1J57" hidden="1">Sheet1!$A$1:$J$57</definedName>
+    <definedName name="_xlchart.v1.0" hidden="1">Sheet1!$E$1</definedName>
+    <definedName name="_xlchart.v1.1" hidden="1">Sheet1!$E$2:$E$51</definedName>
+    <definedName name="_xlchart.v1.10" hidden="1">Sheet1!$F$2:$F$51</definedName>
+    <definedName name="_xlchart.v1.11" hidden="1">Sheet1!$G$1</definedName>
+    <definedName name="_xlchart.v1.12" hidden="1">Sheet1!$G$2:$G$51</definedName>
+    <definedName name="_xlchart.v1.13" hidden="1">Sheet1!$G$2:$G$51</definedName>
+    <definedName name="_xlchart.v1.14" hidden="1">Sheet1!$G$2:$G$51</definedName>
+    <definedName name="_xlchart.v1.15" hidden="1">Sheet1!$G$2:$G$51</definedName>
+    <definedName name="_xlchart.v1.16" hidden="1">Sheet1!$G$2:$G$51</definedName>
+    <definedName name="_xlchart.v1.17" hidden="1">Sheet1!$E$1</definedName>
+    <definedName name="_xlchart.v1.18" hidden="1">Sheet1!$E$2:$E$51</definedName>
+    <definedName name="_xlchart.v1.2" hidden="1">Sheet1!$A$2:$B$51</definedName>
+    <definedName name="_xlchart.v1.3" hidden="1">Sheet1!$C$1</definedName>
+    <definedName name="_xlchart.v1.4" hidden="1">Sheet1!$C$2:$C$51</definedName>
+    <definedName name="_xlchart.v1.5" hidden="1">Sheet1!$D$1</definedName>
+    <definedName name="_xlchart.v1.6" hidden="1">Sheet1!$D$2:$D$51</definedName>
+    <definedName name="_xlchart.v1.7" hidden="1">Sheet1!$E$1</definedName>
+    <definedName name="_xlchart.v1.8" hidden="1">Sheet1!$E$2:$E$51</definedName>
+    <definedName name="_xlchart.v1.9" hidden="1">Sheet1!$F$1</definedName>
+    <definedName name="_xlcn.WorksheetConnection_Sheet1A1J571" hidden="1">Sheet1!$A$1:$J$57</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <pivotCaches>
-    <pivotCache cacheId="67" r:id="rId3"/>
+    <pivotCache cacheId="67" r:id="rId4"/>
   </pivotCaches>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -62,7 +82,7 @@
     <extLst>
       <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{DE250136-89BD-433C-8126-D09CA5730AF9}">
         <x15:connection id="Range" autoDelete="1">
-          <x15:rangePr sourceName="_xlcn.WorksheetConnection_Sheet1A1J57"/>
+          <x15:rangePr sourceName="_xlcn.WorksheetConnection_Sheet1A1J571"/>
         </x15:connection>
       </ext>
     </extLst>
@@ -71,7 +91,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="442" uniqueCount="46">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="446" uniqueCount="50">
   <si>
     <t>Year</t>
   </si>
@@ -210,6 +230,18 @@
   <si>
     <t>Sum of Rainy Days</t>
   </si>
+  <si>
+    <t>It shows the highest rainfallduring the year and lowest rainfall</t>
+  </si>
+  <si>
+    <t>It shows the range of Temperature from highest to lowest</t>
+  </si>
+  <si>
+    <t xml:space="preserve">It shows how many times  did it rain a year </t>
+  </si>
+  <si>
+    <t>IT summarize the average of temperature,humidity,rainy days</t>
+  </si>
 </sst>
 </file>
 
@@ -296,6 +328,4132 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="en-US"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="en-US"/>
+              <a:t>Average</a:t>
+            </a:r>
+            <a:r>
+              <a:rPr lang="en-US" baseline="0"/>
+              <a:t> of Temperature,Humidity and Rainy days,</a:t>
+            </a:r>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="en-KE"/>
+        </a:p>
+      </c:txPr>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:layout/>
+      <c:barChart>
+        <c:barDir val="col"/>
+        <c:grouping val="stacked"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:spPr>
+            <a:solidFill>
+              <a:schemeClr val="accent1"/>
+            </a:solidFill>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:invertIfNegative val="0"/>
+          <c:val>
+            <c:numRef>
+              <c:f>Sheet1!$E$55:$G$55</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="3"/>
+                <c:pt idx="0">
+                  <c:v>22.923999999999999</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>71.959999999999994</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>9.6999999999999993</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-01B6-4A4E-95F8-06F69BCE6106}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:gapWidth val="150"/>
+        <c:overlap val="100"/>
+        <c:axId val="1726420480"/>
+        <c:axId val="1726432000"/>
+      </c:barChart>
+      <c:catAx>
+        <c:axId val="1726420480"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="15000"/>
+                <a:lumOff val="85000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-KE"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="1726432000"/>
+        <c:crosses val="autoZero"/>
+        <c:auto val="1"/>
+        <c:lblAlgn val="ctr"/>
+        <c:lblOffset val="100"/>
+        <c:noMultiLvlLbl val="0"/>
+      </c:catAx>
+      <c:valAx>
+        <c:axId val="1726432000"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-KE"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="1726420480"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="between"/>
+      </c:valAx>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+    </c:plotArea>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
+    <c:extLst>
+      <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
+        <c16r3:dataDisplayOptions16>
+          <c16r3:dispNaAsBlank val="1"/>
+        </c16r3:dataDisplayOptions16>
+      </c:ext>
+    </c:extLst>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:schemeClr val="bg1"/>
+    </a:solidFill>
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:solidFill>
+        <a:schemeClr val="tx1">
+          <a:lumMod val="15000"/>
+          <a:lumOff val="85000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+    <a:effectLst/>
+  </c:spPr>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr/>
+      </a:pPr>
+      <a:endParaRPr lang="en-KE"/>
+    </a:p>
+  </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="en-US"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:chart>
+    <c:title>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="en-KE"/>
+        </a:p>
+      </c:txPr>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:layout/>
+      <c:barChart>
+        <c:barDir val="col"/>
+        <c:grouping val="stacked"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>Sheet1!$D$1</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Rainfall(mm)</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:schemeClr val="accent1"/>
+            </a:solidFill>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:invertIfNegative val="0"/>
+          <c:val>
+            <c:numRef>
+              <c:f>Sheet1!$D$2:$D$51</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="50"/>
+                <c:pt idx="0">
+                  <c:v>45</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>32</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>95</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>180</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>140</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>35</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>20</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>25</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>30</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>90</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>210</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>160</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>50</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>28</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>120</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>190</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>155</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>140</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>18</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>22</c:v>
+                </c:pt>
+                <c:pt idx="20">
+                  <c:v>35</c:v>
+                </c:pt>
+                <c:pt idx="21">
+                  <c:v>105</c:v>
+                </c:pt>
+                <c:pt idx="22">
+                  <c:v>175</c:v>
+                </c:pt>
+                <c:pt idx="23">
+                  <c:v>130</c:v>
+                </c:pt>
+                <c:pt idx="24">
+                  <c:v>42</c:v>
+                </c:pt>
+                <c:pt idx="25">
+                  <c:v>30</c:v>
+                </c:pt>
+                <c:pt idx="26">
+                  <c:v>100</c:v>
+                </c:pt>
+                <c:pt idx="27">
+                  <c:v>165</c:v>
+                </c:pt>
+                <c:pt idx="28">
+                  <c:v>135</c:v>
+                </c:pt>
+                <c:pt idx="29">
+                  <c:v>38</c:v>
+                </c:pt>
+                <c:pt idx="30">
+                  <c:v>19</c:v>
+                </c:pt>
+                <c:pt idx="31">
+                  <c:v>24</c:v>
+                </c:pt>
+                <c:pt idx="32">
+                  <c:v>33</c:v>
+                </c:pt>
+                <c:pt idx="33">
+                  <c:v>38</c:v>
+                </c:pt>
+                <c:pt idx="34">
+                  <c:v>195</c:v>
+                </c:pt>
+                <c:pt idx="35">
+                  <c:v>145</c:v>
+                </c:pt>
+                <c:pt idx="36">
+                  <c:v>60</c:v>
+                </c:pt>
+                <c:pt idx="37">
+                  <c:v>55</c:v>
+                </c:pt>
+                <c:pt idx="38">
+                  <c:v>160</c:v>
+                </c:pt>
+                <c:pt idx="39">
+                  <c:v>220</c:v>
+                </c:pt>
+                <c:pt idx="40">
+                  <c:v>185</c:v>
+                </c:pt>
+                <c:pt idx="41">
+                  <c:v>110</c:v>
+                </c:pt>
+                <c:pt idx="42">
+                  <c:v>90</c:v>
+                </c:pt>
+                <c:pt idx="43">
+                  <c:v>105</c:v>
+                </c:pt>
+                <c:pt idx="44">
+                  <c:v>130</c:v>
+                </c:pt>
+                <c:pt idx="45">
+                  <c:v>190</c:v>
+                </c:pt>
+                <c:pt idx="46">
+                  <c:v>260</c:v>
+                </c:pt>
+                <c:pt idx="47">
+                  <c:v>205</c:v>
+                </c:pt>
+                <c:pt idx="48">
+                  <c:v>75</c:v>
+                </c:pt>
+                <c:pt idx="49">
+                  <c:v>65</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-F3AE-4484-B648-50CF68891B47}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:gapWidth val="150"/>
+        <c:overlap val="100"/>
+        <c:axId val="1835545728"/>
+        <c:axId val="1835543328"/>
+      </c:barChart>
+      <c:catAx>
+        <c:axId val="1835545728"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="15000"/>
+                <a:lumOff val="85000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-KE"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="1835543328"/>
+        <c:crosses val="autoZero"/>
+        <c:auto val="1"/>
+        <c:lblAlgn val="ctr"/>
+        <c:lblOffset val="100"/>
+        <c:noMultiLvlLbl val="0"/>
+      </c:catAx>
+      <c:valAx>
+        <c:axId val="1835543328"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-KE"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="1835545728"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="between"/>
+      </c:valAx>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+    </c:plotArea>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
+    <c:extLst>
+      <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
+        <c16r3:dataDisplayOptions16>
+          <c16r3:dispNaAsBlank val="1"/>
+        </c16r3:dataDisplayOptions16>
+      </c:ext>
+    </c:extLst>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:schemeClr val="bg1"/>
+    </a:solidFill>
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:solidFill>
+        <a:schemeClr val="tx1">
+          <a:lumMod val="15000"/>
+          <a:lumOff val="85000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+    <a:effectLst/>
+  </c:spPr>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr/>
+      </a:pPr>
+      <a:endParaRPr lang="en-KE"/>
+    </a:p>
+  </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="en-US"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="en-US"/>
+              <a:t>Average</a:t>
+            </a:r>
+            <a:r>
+              <a:rPr lang="en-US" baseline="0"/>
+              <a:t> of Temperature,Humidity and Rainy days,</a:t>
+            </a:r>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="en-US"/>
+        </a:p>
+      </c:txPr>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:layout/>
+      <c:barChart>
+        <c:barDir val="col"/>
+        <c:grouping val="stacked"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:spPr>
+            <a:solidFill>
+              <a:schemeClr val="accent1"/>
+            </a:solidFill>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:invertIfNegative val="0"/>
+          <c:val>
+            <c:numRef>
+              <c:f>Sheet1!$E$55:$G$55</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="3"/>
+                <c:pt idx="0">
+                  <c:v>22.923999999999999</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>71.959999999999994</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>9.6999999999999993</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-2CA9-467F-870B-3BC39BC2A26E}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:gapWidth val="150"/>
+        <c:overlap val="100"/>
+        <c:axId val="1726420480"/>
+        <c:axId val="1726432000"/>
+      </c:barChart>
+      <c:catAx>
+        <c:axId val="1726420480"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="15000"/>
+                <a:lumOff val="85000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-KE"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="1726432000"/>
+        <c:crosses val="autoZero"/>
+        <c:auto val="1"/>
+        <c:lblAlgn val="ctr"/>
+        <c:lblOffset val="100"/>
+        <c:noMultiLvlLbl val="0"/>
+      </c:catAx>
+      <c:valAx>
+        <c:axId val="1726432000"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-KE"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="1726420480"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="between"/>
+      </c:valAx>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+    </c:plotArea>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
+    <c:extLst>
+      <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
+        <c16r3:dataDisplayOptions16>
+          <c16r3:dispNaAsBlank val="1"/>
+        </c16r3:dataDisplayOptions16>
+      </c:ext>
+    </c:extLst>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:schemeClr val="bg1"/>
+    </a:solidFill>
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:solidFill>
+        <a:schemeClr val="tx1">
+          <a:lumMod val="15000"/>
+          <a:lumOff val="85000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+    <a:effectLst/>
+  </c:spPr>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr/>
+      </a:pPr>
+      <a:endParaRPr lang="en-KE"/>
+    </a:p>
+  </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/chartEx1.xml><?xml version="1.0" encoding="utf-8"?>
+<cx:chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex">
+  <cx:chartData>
+    <cx:data id="0">
+      <cx:numDim type="val">
+        <cx:f>_xlchart.v1.18</cx:f>
+      </cx:numDim>
+    </cx:data>
+  </cx:chartData>
+  <cx:chart>
+    <cx:title pos="t" align="ctr" overlay="0">
+      <cx:tx>
+        <cx:txData>
+          <cx:v>Temperature(c) of the year</cx:v>
+        </cx:txData>
+      </cx:tx>
+      <cx:txPr>
+        <a:bodyPr spcFirstLastPara="1" vertOverflow="ellipsis" horzOverflow="overflow" wrap="square" lIns="0" tIns="0" rIns="0" bIns="0" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="ctr" rtl="0">
+            <a:defRPr/>
+          </a:pPr>
+          <a:r>
+            <a:rPr lang="en-US" sz="1400" b="0" i="0" u="none" strike="noStrike" baseline="0">
+              <a:solidFill>
+                <a:sysClr val="windowText" lastClr="000000">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:sysClr>
+              </a:solidFill>
+              <a:latin typeface="Calibri" panose="020F0502020204030204"/>
+            </a:rPr>
+            <a:t>Temperature(c) of the year</a:t>
+          </a:r>
+        </a:p>
+      </cx:txPr>
+    </cx:title>
+    <cx:plotArea>
+      <cx:plotAreaRegion>
+        <cx:series layoutId="clusteredColumn" uniqueId="{00000000-000E-4197-B8F8-150D1DE55679}">
+          <cx:tx>
+            <cx:txData>
+              <cx:f>_xlchart.v1.17</cx:f>
+              <cx:v>Temp(c)</cx:v>
+            </cx:txData>
+          </cx:tx>
+          <cx:dataId val="0"/>
+          <cx:layoutPr>
+            <cx:binning intervalClosed="r"/>
+          </cx:layoutPr>
+        </cx:series>
+      </cx:plotAreaRegion>
+      <cx:axis id="0">
+        <cx:catScaling gapWidth="0"/>
+        <cx:tickLabels/>
+      </cx:axis>
+      <cx:axis id="1">
+        <cx:valScaling/>
+        <cx:majorGridlines/>
+        <cx:tickLabels/>
+      </cx:axis>
+    </cx:plotArea>
+  </cx:chart>
+</cx:chartSpace>
+</file>
+
+<file path=xl/charts/chartEx2.xml><?xml version="1.0" encoding="utf-8"?>
+<cx:chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex">
+  <cx:chartData>
+    <cx:data id="0">
+      <cx:numDim type="val">
+        <cx:f>_xlchart.v1.16</cx:f>
+      </cx:numDim>
+    </cx:data>
+  </cx:chartData>
+  <cx:chart>
+    <cx:title pos="t" align="ctr" overlay="0">
+      <cx:tx>
+        <cx:txData>
+          <cx:v>Rainy days</cx:v>
+        </cx:txData>
+      </cx:tx>
+      <cx:txPr>
+        <a:bodyPr spcFirstLastPara="1" vertOverflow="ellipsis" horzOverflow="overflow" wrap="square" lIns="0" tIns="0" rIns="0" bIns="0" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="ctr" rtl="0">
+            <a:defRPr/>
+          </a:pPr>
+          <a:r>
+            <a:rPr lang="en-US" sz="1400" b="0" i="0" u="none" strike="noStrike" baseline="0">
+              <a:solidFill>
+                <a:sysClr val="windowText" lastClr="000000">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:sysClr>
+              </a:solidFill>
+              <a:latin typeface="Calibri" panose="020F0502020204030204"/>
+            </a:rPr>
+            <a:t>Rainy days</a:t>
+          </a:r>
+        </a:p>
+      </cx:txPr>
+    </cx:title>
+    <cx:plotArea>
+      <cx:plotAreaRegion>
+        <cx:series layoutId="clusteredColumn" uniqueId="{00000000-618C-477F-8FE2-EFD4B1F9AC0D}">
+          <cx:dataId val="0"/>
+          <cx:layoutPr>
+            <cx:binning intervalClosed="r"/>
+          </cx:layoutPr>
+        </cx:series>
+      </cx:plotAreaRegion>
+      <cx:axis id="0">
+        <cx:catScaling gapWidth="0"/>
+        <cx:tickLabels/>
+      </cx:axis>
+      <cx:axis id="1">
+        <cx:valScaling/>
+        <cx:majorGridlines/>
+        <cx:tickLabels/>
+      </cx:axis>
+    </cx:plotArea>
+  </cx:chart>
+</cx:chartSpace>
+</file>
+
+<file path=xl/charts/colors1.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent2"/>
+  <a:schemeClr val="accent3"/>
+  <a:schemeClr val="accent4"/>
+  <a:schemeClr val="accent5"/>
+  <a:schemeClr val="accent6"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
+</file>
+
+<file path=xl/charts/colors2.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent2"/>
+  <a:schemeClr val="accent3"/>
+  <a:schemeClr val="accent4"/>
+  <a:schemeClr val="accent5"/>
+  <a:schemeClr val="accent6"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
+</file>
+
+<file path=xl/charts/colors3.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent2"/>
+  <a:schemeClr val="accent3"/>
+  <a:schemeClr val="accent4"/>
+  <a:schemeClr val="accent5"/>
+  <a:schemeClr val="accent6"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
+</file>
+
+<file path=xl/charts/colors4.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent2"/>
+  <a:schemeClr val="accent3"/>
+  <a:schemeClr val="accent4"/>
+  <a:schemeClr val="accent5"/>
+  <a:schemeClr val="accent6"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
+</file>
+
+<file path=xl/charts/colors5.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent2"/>
+  <a:schemeClr val="accent3"/>
+  <a:schemeClr val="accent4"/>
+  <a:schemeClr val="accent5"/>
+  <a:schemeClr val="accent6"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
+</file>
+
+<file path=xl/charts/style1.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="297">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="28575" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="75000"/>
+          <a:lumOff val="25000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="5000"/>
+            <a:lumOff val="95000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="50000"/>
+            <a:lumOff val="50000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:legend>
+  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1400" b="0" kern="1200" spc="0" baseline="0"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:prstDash val="sysDot"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
+<file path=xl/charts/style2.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="297">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="28575" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="75000"/>
+          <a:lumOff val="25000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="5000"/>
+            <a:lumOff val="95000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="50000"/>
+            <a:lumOff val="50000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:legend>
+  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1400" b="0" kern="1200" spc="0" baseline="0"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:prstDash val="sysDot"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
+<file path=xl/charts/style3.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="366">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="1000"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="phClr"/>
+      </a:solidFill>
+    </cs:spPr>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="phClr"/>
+      </a:solidFill>
+    </cs:spPr>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="28575" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="phClr"/>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="lt1"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="28575" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="65000"/>
+          <a:lumOff val="35000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="75000"/>
+            <a:lumOff val="25000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900"/>
+  </cs:legend>
+  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat">
+        <a:solidFill>
+          <a:srgbClr val="D9D9D9"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1400"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:prstDash val="sysDash"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
+<file path=xl/charts/style4.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="366">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="1000"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="phClr"/>
+      </a:solidFill>
+    </cs:spPr>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="phClr"/>
+      </a:solidFill>
+    </cs:spPr>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="28575" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="phClr"/>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="lt1"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="28575" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="65000"/>
+          <a:lumOff val="35000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="75000"/>
+            <a:lumOff val="25000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900"/>
+  </cs:legend>
+  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat">
+        <a:solidFill>
+          <a:srgbClr val="D9D9D9"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1400"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:prstDash val="sysDash"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
+<file path=xl/charts/style5.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="297">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="28575" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="75000"/>
+          <a:lumOff val="25000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="5000"/>
+            <a:lumOff val="95000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="50000"/>
+            <a:lumOff val="50000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:legend>
+  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1400" b="0" kern="1200" spc="0" baseline="0"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:prstDash val="sysDot"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>396240</xdr:colOff>
+      <xdr:row>47</xdr:row>
+      <xdr:rowOff>80010</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>1043940</xdr:colOff>
+      <xdr:row>62</xdr:row>
+      <xdr:rowOff>80010</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="14" name="Chart 13">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{8A8744E5-E22E-B534-1855-AE44654B3280}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>304800</xdr:colOff>
+      <xdr:row>15</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="2" name="Chart 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{9EA7378D-E9D4-4A19-ABF5-3D4D996C4EFF}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr>
+          <a:graphicFrameLocks/>
+        </xdr:cNvGraphicFramePr>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>18</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>304800</xdr:colOff>
+      <xdr:row>33</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:to>
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+      <mc:Choice xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" Requires="cx1">
+        <xdr:graphicFrame macro="">
+          <xdr:nvGraphicFramePr>
+            <xdr:cNvPr id="3" name="Chart 2">
+              <a:extLst>
+                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{65656355-6C4B-44FD-A1A6-C6C11ACE1292}"/>
+                </a:ext>
+              </a:extLst>
+            </xdr:cNvPr>
+            <xdr:cNvGraphicFramePr/>
+          </xdr:nvGraphicFramePr>
+          <xdr:xfrm>
+            <a:off x="0" y="0"/>
+            <a:ext cx="0" cy="0"/>
+          </xdr:xfrm>
+          <a:graphic>
+            <a:graphicData uri="http://schemas.microsoft.com/office/drawing/2014/chartex">
+              <cx:chart xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
+            </a:graphicData>
+          </a:graphic>
+        </xdr:graphicFrame>
+      </mc:Choice>
+      <mc:Fallback>
+        <xdr:sp macro="" textlink="">
+          <xdr:nvSpPr>
+            <xdr:cNvPr id="0" name=""/>
+            <xdr:cNvSpPr>
+              <a:spLocks noTextEdit="1"/>
+            </xdr:cNvSpPr>
+          </xdr:nvSpPr>
+          <xdr:spPr>
+            <a:xfrm>
+              <a:off x="0" y="3291840"/>
+              <a:ext cx="4572000" cy="2743200"/>
+            </a:xfrm>
+            <a:prstGeom prst="rect">
+              <a:avLst/>
+            </a:prstGeom>
+            <a:solidFill>
+              <a:prstClr val="white"/>
+            </a:solidFill>
+            <a:ln w="1">
+              <a:solidFill>
+                <a:prstClr val="green"/>
+              </a:solidFill>
+            </a:ln>
+          </xdr:spPr>
+          <xdr:txBody>
+            <a:bodyPr vertOverflow="clip" horzOverflow="clip"/>
+            <a:lstStyle/>
+            <a:p>
+              <a:r>
+                <a:rPr lang="en-KE" sz="1100"/>
+                <a:t>This chart isn't available in your version of Excel.
+Editing this shape or saving this workbook into a different file format will permanently break the chart.</a:t>
+              </a:r>
+            </a:p>
+          </xdr:txBody>
+        </xdr:sp>
+      </mc:Fallback>
+    </mc:AlternateContent>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>2</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>15</xdr:col>
+      <xdr:colOff>304800</xdr:colOff>
+      <xdr:row>17</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:to>
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+      <mc:Choice xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" Requires="cx1">
+        <xdr:graphicFrame macro="">
+          <xdr:nvGraphicFramePr>
+            <xdr:cNvPr id="4" name="Chart 3">
+              <a:extLst>
+                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{640231B2-71A1-4603-B54C-6A2651C8291E}"/>
+                </a:ext>
+              </a:extLst>
+            </xdr:cNvPr>
+            <xdr:cNvGraphicFramePr/>
+          </xdr:nvGraphicFramePr>
+          <xdr:xfrm>
+            <a:off x="0" y="0"/>
+            <a:ext cx="0" cy="0"/>
+          </xdr:xfrm>
+          <a:graphic>
+            <a:graphicData uri="http://schemas.microsoft.com/office/drawing/2014/chartex">
+              <cx:chart xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId3"/>
+            </a:graphicData>
+          </a:graphic>
+        </xdr:graphicFrame>
+      </mc:Choice>
+      <mc:Fallback>
+        <xdr:sp macro="" textlink="">
+          <xdr:nvSpPr>
+            <xdr:cNvPr id="0" name=""/>
+            <xdr:cNvSpPr>
+              <a:spLocks noTextEdit="1"/>
+            </xdr:cNvSpPr>
+          </xdr:nvSpPr>
+          <xdr:spPr>
+            <a:xfrm>
+              <a:off x="4876800" y="365760"/>
+              <a:ext cx="4572000" cy="2743200"/>
+            </a:xfrm>
+            <a:prstGeom prst="rect">
+              <a:avLst/>
+            </a:prstGeom>
+            <a:solidFill>
+              <a:prstClr val="white"/>
+            </a:solidFill>
+            <a:ln w="1">
+              <a:solidFill>
+                <a:prstClr val="green"/>
+              </a:solidFill>
+            </a:ln>
+          </xdr:spPr>
+          <xdr:txBody>
+            <a:bodyPr vertOverflow="clip" horzOverflow="clip"/>
+            <a:lstStyle/>
+            <a:p>
+              <a:r>
+                <a:rPr lang="en-KE" sz="1100"/>
+                <a:t>This chart isn't available in your version of Excel.
+Editing this shape or saving this workbook into a different file format will permanently break the chart.</a:t>
+              </a:r>
+            </a:p>
+          </xdr:txBody>
+        </xdr:sp>
+      </mc:Fallback>
+    </mc:AlternateContent>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>21</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>15</xdr:col>
+      <xdr:colOff>304800</xdr:colOff>
+      <xdr:row>36</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="5" name="Chart 4">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{E5BB4B40-8AF3-4930-97CC-6FABD2E50C97}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr>
+          <a:graphicFrameLocks/>
+        </xdr:cNvGraphicFramePr>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId4"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
 </file>
 
 <file path=xl/pivotCache/pivotCacheDefinition1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -6142,5 +10300,37 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+  <drawing r:id="rId2"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{86A17BE4-581D-454C-B271-46213657A423}">
+  <dimension ref="A16:I37"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetData>
+    <row r="16" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A16" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="18" spans="9:9" x14ac:dyDescent="0.3">
+      <c r="I18" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="34" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A34" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="37" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="I37" t="s">
+        <v>49</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>